<commit_message>
fix(routing): correct bicycle slope units
</commit_message>
<xml_diff>
--- a/tests/referral/data/result_conf_all.xlsx
+++ b/tests/referral/data/result_conf_all.xlsx
@@ -407,7 +407,7 @@
         <v>52</v>
       </c>
       <c r="F2">
-        <v>686</v>
+        <v>703</v>
       </c>
     </row>
     <row r="3">
@@ -431,7 +431,7 @@
         <v>160</v>
       </c>
       <c r="F3">
-        <v>1277</v>
+        <v>1294</v>
       </c>
     </row>
     <row r="4">
@@ -455,7 +455,7 @@
         <v>75</v>
       </c>
       <c r="F4">
-        <v>702</v>
+        <v>719</v>
       </c>
     </row>
     <row r="5">
@@ -479,7 +479,7 @@
         <v>96</v>
       </c>
       <c r="F5">
-        <v>721</v>
+        <v>738</v>
       </c>
     </row>
     <row r="6">
@@ -503,7 +503,7 @@
         <v>124</v>
       </c>
       <c r="F6">
-        <v>751</v>
+        <v>769</v>
       </c>
     </row>
     <row r="7">
@@ -527,7 +527,7 @@
         <v>73</v>
       </c>
       <c r="F7">
-        <v>704</v>
+        <v>721</v>
       </c>
     </row>
     <row r="8">
@@ -551,7 +551,7 @@
         <v>134</v>
       </c>
       <c r="F8">
-        <v>1064</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="9">
@@ -575,7 +575,7 @@
         <v>65</v>
       </c>
       <c r="F9">
-        <v>703</v>
+        <v>720</v>
       </c>
     </row>
     <row r="10">
@@ -599,7 +599,7 @@
         <v>87</v>
       </c>
       <c r="F10">
-        <v>781</v>
+        <v>798</v>
       </c>
     </row>
     <row r="11">
@@ -620,10 +620,10 @@
         </is>
       </c>
       <c r="E11">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="F11">
-        <v>632</v>
+        <v>603</v>
       </c>
     </row>
     <row r="12">
@@ -836,10 +836,10 @@
         </is>
       </c>
       <c r="E20">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="F20">
-        <v>1199</v>
+        <v>1184</v>
       </c>
     </row>
     <row r="21">
@@ -1052,10 +1052,10 @@
         </is>
       </c>
       <c r="E29">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="F29">
-        <v>647</v>
+        <v>619</v>
       </c>
     </row>
     <row r="30">
@@ -1268,10 +1268,10 @@
         </is>
       </c>
       <c r="E38">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="F38">
-        <v>666</v>
+        <v>638</v>
       </c>
     </row>
     <row r="39">
@@ -1484,10 +1484,10 @@
         </is>
       </c>
       <c r="E47">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="F47">
-        <v>697</v>
+        <v>681</v>
       </c>
     </row>
     <row r="48">
@@ -1700,10 +1700,10 @@
         </is>
       </c>
       <c r="E56">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="F56">
-        <v>650</v>
+        <v>634</v>
       </c>
     </row>
     <row r="57">
@@ -1916,10 +1916,10 @@
         </is>
       </c>
       <c r="E65">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="F65">
-        <v>1006</v>
+        <v>991</v>
       </c>
     </row>
     <row r="66">
@@ -2132,10 +2132,10 @@
         </is>
       </c>
       <c r="E74">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F74">
-        <v>648</v>
+        <v>633</v>
       </c>
     </row>
     <row r="75">
@@ -2348,10 +2348,10 @@
         </is>
       </c>
       <c r="E83">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F83">
-        <v>734</v>
+        <v>719</v>
       </c>
     </row>
     <row r="84">

</xml_diff>

<commit_message>
fix(mobility): reject non-finite bicycle slopes
</commit_message>
<xml_diff>
--- a/tests/referral/data/result_conf_all.xlsx
+++ b/tests/referral/data/result_conf_all.xlsx
@@ -623,7 +623,7 @@
         <v>48</v>
       </c>
       <c r="F11">
-        <v>603</v>
+        <v>634</v>
       </c>
     </row>
     <row r="12">
@@ -836,10 +836,10 @@
         </is>
       </c>
       <c r="E20">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="F20">
-        <v>1184</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="21">
@@ -1055,7 +1055,7 @@
         <v>71</v>
       </c>
       <c r="F29">
-        <v>619</v>
+        <v>650</v>
       </c>
     </row>
     <row r="30">
@@ -1271,7 +1271,7 @@
         <v>92</v>
       </c>
       <c r="F38">
-        <v>638</v>
+        <v>669</v>
       </c>
     </row>
     <row r="39">
@@ -1484,10 +1484,10 @@
         </is>
       </c>
       <c r="E47">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="F47">
-        <v>681</v>
+        <v>709</v>
       </c>
     </row>
     <row r="48">
@@ -1700,10 +1700,10 @@
         </is>
       </c>
       <c r="E56">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="F56">
-        <v>634</v>
+        <v>661</v>
       </c>
     </row>
     <row r="57">
@@ -1916,10 +1916,10 @@
         </is>
       </c>
       <c r="E65">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="F65">
-        <v>991</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="66">
@@ -2132,10 +2132,10 @@
         </is>
       </c>
       <c r="E74">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="F74">
-        <v>633</v>
+        <v>660</v>
       </c>
     </row>
     <row r="75">
@@ -2348,10 +2348,10 @@
         </is>
       </c>
       <c r="E83">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="F83">
-        <v>719</v>
+        <v>746</v>
       </c>
     </row>
     <row r="84">

</xml_diff>